<commit_message>
Add Discord links, accessory FAQ, filter tooltips + favicon; refresh Blackarrow gear data
</commit_message>
<xml_diff>
--- a/Class_Gear_and_Gem_Database.xlsx
+++ b/Class_Gear_and_Gem_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orien\Desktop\mistfall calc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DBAB0F1-93DD-4806-A416-0031FA731D46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0C50F33-0CBA-447C-89B5-665ECBC5F5EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="180" yWindow="315" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gear Database" sheetId="1" r:id="rId1"/>
@@ -11123,7 +11123,7 @@
         <v>61</v>
       </c>
       <c r="B361" s="17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C361" s="4" t="s">
         <v>42</v>
@@ -11148,8 +11148,8 @@
       <c r="A362" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="B362" s="18" t="s">
-        <v>74</v>
+      <c r="B362" s="17" t="s">
+        <v>73</v>
       </c>
       <c r="C362" s="15" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
Seer True Prayer Miter: Change Creation socket to Triangle T2
</commit_message>
<xml_diff>
--- a/Class_Gear_and_Gem_Database.xlsx
+++ b/Class_Gear_and_Gem_Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orien\Desktop\mistfall calc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0C50F33-0CBA-447C-89B5-665ECBC5F5EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD169E3-4EC3-4CB8-A4D1-D7F739F0DB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2376,7 +2376,7 @@
         <v>20</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="G24" s="4" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Rarity preference per slot, on-demand show-more builds, empty socket labels; Seer socket fix
</commit_message>
<xml_diff>
--- a/Class_Gear_and_Gem_Database.xlsx
+++ b/Class_Gear_and_Gem_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orien\Desktop\mistfall calc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD169E3-4EC3-4CB8-A4D1-D7F739F0DB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8807549-8E05-4B4E-BAE0-4BDBBD56A970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9600" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gear Database" sheetId="1" r:id="rId1"/>
@@ -9237,7 +9237,7 @@
         <v>343</v>
       </c>
       <c r="F288" s="27" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="G288" s="27" t="s">
         <v>26</v>

</xml_diff>